<commit_message>
Add refundable SR&ED ITC portion to the credits calculation
New optional intake field sred_itc_refundable (tab 12 row "Refundable
Portion of SR&ED ITC ($)"; template defaults it to the full ITC when the
enhanced 35% rate applies). Non-refundable credits are applied against
Part I tax first; the refundable portion covers any remaining Part I
tax and the rest is paid in cash (s.127.1) and included in the year-end
position, with a flag that it depends on CRA accepting the claim. A
refundable portion above the total ITC raises ValueError.

Defaults to 0 when absent, preserving the conservative behaviour. No
expected regression value changes: the Northern Peak fixture is marked
fully refundable but its Part I tax exceeds its credits.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/clients/_template/CCPC_Tax_Planning_Intake_Workbook.xlsx
+++ b/clients/_template/CCPC_Tax_Planning_Intake_Workbook.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/207c16c34f2daf9f/Google Drive Docs/Biz Infograph/Claude/tax-planning-agent_rate_llm/clients/_template/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="11_44A903A2E52269CB727786B3BF84C54966D86C59" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F7FF892A-103F-4FE3-A81A-DF0210076B6E}"/>
+  <xr:revisionPtr revIDLastSave="6" documentId="11_44A903A2E52269CB727786B3BF84C54966D86C59" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{16DF8D4F-B7D7-4381-B990-F12280691290}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="658" uniqueCount="536">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="660" uniqueCount="538">
   <si>
     <t>CCPC Corporate Tax Planning &amp; Compliance Intake Workbook</t>
   </si>
@@ -1657,6 +1657,12 @@
   </si>
   <si>
     <t>Connected (sister corp under common control, s.186(4)): deductible under s.112, NOT active business income. Part IV = this corp's share of the payer's dividend refund - enter it in the holdco section below.</t>
+  </si>
+  <si>
+    <t>Refundable Portion of SR&amp;ED ITC ($)</t>
+  </si>
+  <si>
+    <t>Cash-refundable part of the ITC (s.127.1). Defaults to the full ITC when the enhanced 35% rate applies (current expenditures of a CCPC under the expenditure limit). Overwrite with the actual refundable amount if part is non-refundable.</t>
   </si>
 </sst>
 </file>
@@ -2037,15 +2043,15 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -2155,6 +2161,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2668,11 +2678,6 @@
     </row>
   </sheetData>
   <mergeCells count="21">
-    <mergeCell ref="A8:D8"/>
-    <mergeCell ref="A22:D22"/>
-    <mergeCell ref="A4:D4"/>
-    <mergeCell ref="B29:D29"/>
-    <mergeCell ref="B28:D28"/>
     <mergeCell ref="A31:D31"/>
     <mergeCell ref="A48:D48"/>
     <mergeCell ref="B24:D24"/>
@@ -2689,6 +2694,11 @@
     <mergeCell ref="A15:D16"/>
     <mergeCell ref="A2:D2"/>
     <mergeCell ref="A11:D12"/>
+    <mergeCell ref="A8:D8"/>
+    <mergeCell ref="A22:D22"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="B29:D29"/>
+    <mergeCell ref="B28:D28"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -3644,7 +3654,7 @@
       <c r="C8" s="11"/>
     </row>
     <row r="9" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="66" t="s">
+      <c r="A9" s="65" t="s">
         <v>392</v>
       </c>
       <c r="B9" s="64"/>
@@ -3684,7 +3694,7 @@
       <c r="C13" s="11"/>
     </row>
     <row r="14" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="66" t="s">
+      <c r="A14" s="65" t="s">
         <v>397</v>
       </c>
       <c r="B14" s="64"/>
@@ -3716,7 +3726,7 @@
       <c r="C17" s="11"/>
     </row>
     <row r="18" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="66" t="s">
+      <c r="A18" s="65" t="s">
         <v>400</v>
       </c>
       <c r="B18" s="64"/>
@@ -3783,7 +3793,7 @@
       <c r="C26" s="11"/>
     </row>
     <row r="27" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="66" t="s">
+      <c r="A27" s="65" t="s">
         <v>408</v>
       </c>
       <c r="B27" s="64"/>
@@ -3812,12 +3822,6 @@
     </row>
   </sheetData>
   <mergeCells count="15">
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A9:D9"/>
-    <mergeCell ref="A16:B16"/>
-    <mergeCell ref="A18:D18"/>
-    <mergeCell ref="A15:B15"/>
-    <mergeCell ref="A7:B7"/>
     <mergeCell ref="A27:D27"/>
     <mergeCell ref="A11:B11"/>
     <mergeCell ref="A3:D3"/>
@@ -3827,6 +3831,12 @@
     <mergeCell ref="A14:D14"/>
     <mergeCell ref="A12:B12"/>
     <mergeCell ref="A4:B4"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A9:D9"/>
+    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="A18:D18"/>
+    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="A7:B7"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -3887,7 +3897,7 @@
       <c r="D3" s="57"/>
     </row>
     <row r="4" spans="1:4" ht="22.35" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="63" t="s">
+      <c r="A4" s="66" t="s">
         <v>413</v>
       </c>
       <c r="B4" s="64"/>
@@ -3951,7 +3961,7 @@
       <c r="C11" s="11"/>
     </row>
     <row r="12" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="66" t="s">
+      <c r="A12" s="65" t="s">
         <v>419</v>
       </c>
       <c r="B12" s="64"/>
@@ -4034,7 +4044,7 @@
       <c r="C21" s="11"/>
     </row>
     <row r="22" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="66" t="s">
+      <c r="A22" s="65" t="s">
         <v>426</v>
       </c>
       <c r="B22" s="64"/>
@@ -4210,12 +4220,20 @@
       </c>
     </row>
     <row r="10" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="11"/>
+      <c r="A10" s="17" t="s">
+        <v>536</v>
+      </c>
       <c r="B10" s="11"/>
-      <c r="C10" s="11"/>
+      <c r="C10" s="16">
+        <f>IF(C8="Yes",C9,0)</f>
+        <v>22750</v>
+      </c>
+      <c r="D10" t="s">
+        <v>537</v>
+      </c>
     </row>
     <row r="11" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="66" t="s">
+      <c r="A11" s="65" t="s">
         <v>441</v>
       </c>
       <c r="B11" s="64"/>
@@ -4223,7 +4241,7 @@
       <c r="D11" s="64"/>
     </row>
     <row r="12" spans="1:4" ht="22.35" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="63" t="s">
+      <c r="A12" s="66" t="s">
         <v>442</v>
       </c>
       <c r="B12" s="64"/>
@@ -4254,7 +4272,7 @@
       <c r="C15" s="11"/>
     </row>
     <row r="16" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="66" t="s">
+      <c r="A16" s="65" t="s">
         <v>446</v>
       </c>
       <c r="B16" s="64"/>
@@ -4300,17 +4318,17 @@
     </row>
   </sheetData>
   <mergeCells count="11">
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="A16:D16"/>
+    <mergeCell ref="A11:D11"/>
+    <mergeCell ref="A8:B8"/>
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A7:B7"/>
     <mergeCell ref="A12:D12"/>
     <mergeCell ref="A3:D3"/>
     <mergeCell ref="A5:B5"/>
-    <mergeCell ref="A13:B13"/>
-    <mergeCell ref="A14:B14"/>
-    <mergeCell ref="A16:D16"/>
-    <mergeCell ref="A11:D11"/>
-    <mergeCell ref="A8:B8"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -5254,7 +5272,7 @@
       <c r="D2" s="57"/>
     </row>
     <row r="4" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="66" t="s">
+      <c r="A4" s="65" t="s">
         <v>46</v>
       </c>
       <c r="B4" s="64"/>
@@ -5302,7 +5320,7 @@
       <c r="B9" s="11"/>
     </row>
     <row r="10" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="66" t="s">
+      <c r="A10" s="65" t="s">
         <v>51</v>
       </c>
       <c r="B10" s="64"/>
@@ -5344,7 +5362,7 @@
       <c r="B14" s="11"/>
     </row>
     <row r="15" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="66" t="s">
+      <c r="A15" s="65" t="s">
         <v>56</v>
       </c>
       <c r="B15" s="64"/>
@@ -5449,7 +5467,7 @@
       <c r="B26" s="11"/>
     </row>
     <row r="27" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="66" t="s">
+      <c r="A27" s="65" t="s">
         <v>68</v>
       </c>
       <c r="B27" s="64"/>
@@ -5526,7 +5544,7 @@
       <c r="B35" s="11"/>
     </row>
     <row r="36" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="66" t="s">
+      <c r="A36" s="65" t="s">
         <v>76</v>
       </c>
       <c r="B36" s="64"/>
@@ -5619,7 +5637,7 @@
       <c r="B46" s="11"/>
     </row>
     <row r="47" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="66" t="s">
+      <c r="A47" s="65" t="s">
         <v>86</v>
       </c>
       <c r="B47" s="64"/>
@@ -5685,7 +5703,7 @@
       <c r="B54" s="11"/>
     </row>
     <row r="55" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A55" s="66" t="s">
+      <c r="A55" s="65" t="s">
         <v>93</v>
       </c>
       <c r="B55" s="64"/>
@@ -5693,7 +5711,7 @@
       <c r="D55" s="64"/>
     </row>
     <row r="56" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A56" s="65" t="str">
+      <c r="A56" s="63" t="str">
         <f>IF(B18&gt;0,"• Passive income is grinding the SBD limit — consider moving investments to a holding company or reducing corporate investment income.","")</f>
         <v>• Passive income is grinding the SBD limit — consider moving investments to a holding company or reducing corporate investment income.</v>
       </c>
@@ -5702,7 +5720,7 @@
       <c r="D56" s="64"/>
     </row>
     <row r="57" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A57" s="65" t="str">
+      <c r="A57" s="63" t="str">
         <f>IF(COUNTIF('8. Shareholders &amp; TOSI'!I5:I20,"Not Excluded - TOSI Risk")&gt;0,"• One or more shareholders flagged for TOSI risk — dividends to them may be taxed at top marginal rate.","")</f>
         <v>• One or more shareholders flagged for TOSI risk — dividends to them may be taxed at top marginal rate.</v>
       </c>
@@ -5711,7 +5729,7 @@
       <c r="D57" s="64"/>
     </row>
     <row r="58" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A58" s="65" t="str">
+      <c r="A58" s="63" t="str">
         <f>IF(B44&gt;0,"• Unused Capital Dividend Account balance — a tax-free capital dividend may be available.","")</f>
         <v>• Unused Capital Dividend Account balance — a tax-free capital dividend may be available.</v>
       </c>
@@ -5720,7 +5738,7 @@
       <c r="D58" s="64"/>
     </row>
     <row r="59" spans="1:4" ht="22.35" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A59" s="63" t="s">
+      <c r="A59" s="66" t="s">
         <v>94</v>
       </c>
       <c r="B59" s="64"/>
@@ -5729,6 +5747,12 @@
     </row>
   </sheetData>
   <mergeCells count="13">
+    <mergeCell ref="A59:D59"/>
+    <mergeCell ref="A57:D57"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A10:D10"/>
+    <mergeCell ref="A36:D36"/>
+    <mergeCell ref="A47:D47"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A56:D56"/>
     <mergeCell ref="A27:D27"/>
@@ -5736,12 +5760,6 @@
     <mergeCell ref="A4:D4"/>
     <mergeCell ref="A55:D55"/>
     <mergeCell ref="A15:D15"/>
-    <mergeCell ref="A59:D59"/>
-    <mergeCell ref="A57:D57"/>
-    <mergeCell ref="A2:D2"/>
-    <mergeCell ref="A10:D10"/>
-    <mergeCell ref="A36:D36"/>
-    <mergeCell ref="A47:D47"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -5989,6 +6007,18 @@
     </row>
   </sheetData>
   <mergeCells count="24">
+    <mergeCell ref="A27:D27"/>
+    <mergeCell ref="A29:B29"/>
+    <mergeCell ref="A19:B19"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A28:B28"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="A25:B25"/>
+    <mergeCell ref="A15:D15"/>
+    <mergeCell ref="A18:B18"/>
+    <mergeCell ref="A12:B12"/>
+    <mergeCell ref="A23:D23"/>
+    <mergeCell ref="A24:B24"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A21:B21"/>
     <mergeCell ref="A5:B5"/>
@@ -6001,18 +6031,6 @@
     <mergeCell ref="A6:B6"/>
     <mergeCell ref="A16:B16"/>
     <mergeCell ref="A7:B7"/>
-    <mergeCell ref="A27:D27"/>
-    <mergeCell ref="A29:B29"/>
-    <mergeCell ref="A19:B19"/>
-    <mergeCell ref="A3:D3"/>
-    <mergeCell ref="A28:B28"/>
-    <mergeCell ref="A13:B13"/>
-    <mergeCell ref="A25:B25"/>
-    <mergeCell ref="A15:D15"/>
-    <mergeCell ref="A18:B18"/>
-    <mergeCell ref="A12:B12"/>
-    <mergeCell ref="A23:D23"/>
-    <mergeCell ref="A24:B24"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -6386,7 +6404,7 @@
       </c>
     </row>
     <row r="4" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="66" t="s">
+      <c r="A4" s="65" t="s">
         <v>154</v>
       </c>
       <c r="B4" s="64"/>
@@ -6431,7 +6449,7 @@
       <c r="B10" s="11"/>
     </row>
     <row r="11" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="66" t="s">
+      <c r="A11" s="65" t="s">
         <v>158</v>
       </c>
       <c r="B11" s="64"/>
@@ -6473,7 +6491,7 @@
       <c r="B16" s="11"/>
     </row>
     <row r="17" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="66" t="s">
+      <c r="A17" s="65" t="s">
         <v>162</v>
       </c>
       <c r="B17" s="64"/>
@@ -6605,7 +6623,7 @@
       <c r="B33" s="11"/>
     </row>
     <row r="34" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="66" t="s">
+      <c r="A34" s="65" t="s">
         <v>178</v>
       </c>
       <c r="B34" s="64"/>
@@ -6725,7 +6743,7 @@
       <c r="B45" s="11"/>
     </row>
     <row r="46" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="66" t="s">
+      <c r="A46" s="65" t="s">
         <v>193</v>
       </c>
       <c r="B46" s="64"/>
@@ -6949,7 +6967,7 @@
       </c>
     </row>
     <row r="4" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="66" t="s">
+      <c r="A4" s="65" t="s">
         <v>224</v>
       </c>
       <c r="B4" s="64"/>
@@ -7054,7 +7072,7 @@
       <c r="B16" s="33"/>
     </row>
     <row r="17" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="66" t="s">
+      <c r="A17" s="65" t="s">
         <v>238</v>
       </c>
       <c r="B17" s="64"/>
@@ -7145,7 +7163,7 @@
       <c r="B28" s="33"/>
     </row>
     <row r="29" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="66" t="s">
+      <c r="A29" s="65" t="s">
         <v>249</v>
       </c>
       <c r="B29" s="64"/>
@@ -7221,7 +7239,7 @@
       <c r="B38" s="33"/>
     </row>
     <row r="39" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="66" t="s">
+      <c r="A39" s="65" t="s">
         <v>257</v>
       </c>
       <c r="B39" s="64"/>
@@ -7293,7 +7311,7 @@
       <c r="D2" s="57"/>
     </row>
     <row r="4" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="66" t="s">
+      <c r="A4" s="65" t="s">
         <v>264</v>
       </c>
       <c r="B4" s="64"/>
@@ -7330,7 +7348,7 @@
       <c r="C7" s="11"/>
     </row>
     <row r="8" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="66" t="s">
+      <c r="A8" s="65" t="s">
         <v>268</v>
       </c>
       <c r="B8" s="64"/>
@@ -7355,7 +7373,7 @@
       <c r="C10" s="11"/>
     </row>
     <row r="11" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="66" t="s">
+      <c r="A11" s="65" t="s">
         <v>271</v>
       </c>
       <c r="B11" s="64"/>
@@ -7380,7 +7398,7 @@
       <c r="C13" s="11"/>
     </row>
     <row r="14" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="66" t="s">
+      <c r="A14" s="65" t="s">
         <v>274</v>
       </c>
       <c r="B14" s="64"/>
@@ -7443,7 +7461,7 @@
       <c r="C20" s="11"/>
     </row>
     <row r="21" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="66" t="s">
+      <c r="A21" s="65" t="s">
         <v>277</v>
       </c>
       <c r="B21" s="64"/>
@@ -7478,7 +7496,7 @@
       <c r="C25" s="11"/>
     </row>
     <row r="26" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="66" t="s">
+      <c r="A26" s="65" t="s">
         <v>278</v>
       </c>
       <c r="B26" s="64"/>
@@ -7517,12 +7535,6 @@
     </row>
   </sheetData>
   <mergeCells count="14">
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A8:D8"/>
-    <mergeCell ref="A4:D4"/>
-    <mergeCell ref="A26:D26"/>
-    <mergeCell ref="A21:D21"/>
-    <mergeCell ref="A5:B5"/>
     <mergeCell ref="A28:B28"/>
     <mergeCell ref="A2:D2"/>
     <mergeCell ref="A11:D11"/>
@@ -7531,6 +7543,12 @@
     <mergeCell ref="A6:B6"/>
     <mergeCell ref="A14:D14"/>
     <mergeCell ref="A12:B12"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A8:D8"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="A26:D26"/>
+    <mergeCell ref="A21:D21"/>
+    <mergeCell ref="A5:B5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Add refundable provincial credit portion to the credits calculation
New optional intake field provincial_credit_refundable (tab 12 row
"Refundable Portion of Provincial Credit ($)", blank in the template
since refundability depends on the program). Non-refundable credits are
applied against Part I tax first; refundable SR&ED, then refundable
provincial, cover any remaining Part I tax and the rest of each is paid
in cash, included in the year-end position, and flagged. A refundable
portion above the provincial credit raises ValueError.

The Northern Peak fixture marks its $9,750 Alberta Innovation Employment
Grant as refundable. No expected regression value changes: its Part I
tax exceeds its credits.

Also documents the OneDrive/Excel AutoSave risk when scripting edits to
the intake workbooks.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/clients/_template/CCPC_Tax_Planning_Intake_Workbook.xlsx
+++ b/clients/_template/CCPC_Tax_Planning_Intake_Workbook.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/207c16c34f2daf9f/Google Drive Docs/Biz Infograph/Claude/tax-planning-agent_rate_llm/clients/_template/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="6" documentId="11_44A903A2E52269CB727786B3BF84C54966D86C59" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{16DF8D4F-B7D7-4381-B990-F12280691290}"/>
+  <xr:revisionPtr revIDLastSave="10" documentId="11_44A903A2E52269CB727786B3BF84C54966D86C59" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2D5721EB-262C-459F-B22F-6D0592710C65}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="660" uniqueCount="538">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="662" uniqueCount="540">
   <si>
     <t>CCPC Corporate Tax Planning &amp; Compliance Intake Workbook</t>
   </si>
@@ -1663,6 +1663,12 @@
   </si>
   <si>
     <t>Cash-refundable part of the ITC (s.127.1). Defaults to the full ITC when the enhanced 35% rate applies (current expenditures of a CCPC under the expenditure limit). Overwrite with the actual refundable amount if part is non-refundable.</t>
+  </si>
+  <si>
+    <t>Refundable Portion of Provincial Credit ($)</t>
+  </si>
+  <si>
+    <t>Part of the provincial credit paid in cash even with no tax owing (e.g., Alberta Innovation Employment Grant). Leave blank if non-refundable - unused amounts then carry forward.</t>
   </si>
 </sst>
 </file>
@@ -2043,15 +2049,15 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -2678,6 +2684,11 @@
     </row>
   </sheetData>
   <mergeCells count="21">
+    <mergeCell ref="A8:D8"/>
+    <mergeCell ref="A22:D22"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="B29:D29"/>
+    <mergeCell ref="B28:D28"/>
     <mergeCell ref="A31:D31"/>
     <mergeCell ref="A48:D48"/>
     <mergeCell ref="B24:D24"/>
@@ -2694,11 +2705,6 @@
     <mergeCell ref="A15:D16"/>
     <mergeCell ref="A2:D2"/>
     <mergeCell ref="A11:D12"/>
-    <mergeCell ref="A8:D8"/>
-    <mergeCell ref="A22:D22"/>
-    <mergeCell ref="A4:D4"/>
-    <mergeCell ref="B29:D29"/>
-    <mergeCell ref="B28:D28"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -3654,7 +3660,7 @@
       <c r="C8" s="11"/>
     </row>
     <row r="9" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="65" t="s">
+      <c r="A9" s="66" t="s">
         <v>392</v>
       </c>
       <c r="B9" s="64"/>
@@ -3694,7 +3700,7 @@
       <c r="C13" s="11"/>
     </row>
     <row r="14" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="65" t="s">
+      <c r="A14" s="66" t="s">
         <v>397</v>
       </c>
       <c r="B14" s="64"/>
@@ -3726,7 +3732,7 @@
       <c r="C17" s="11"/>
     </row>
     <row r="18" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="65" t="s">
+      <c r="A18" s="66" t="s">
         <v>400</v>
       </c>
       <c r="B18" s="64"/>
@@ -3793,7 +3799,7 @@
       <c r="C26" s="11"/>
     </row>
     <row r="27" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="65" t="s">
+      <c r="A27" s="66" t="s">
         <v>408</v>
       </c>
       <c r="B27" s="64"/>
@@ -3822,6 +3828,12 @@
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A9:D9"/>
+    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="A18:D18"/>
+    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="A7:B7"/>
     <mergeCell ref="A27:D27"/>
     <mergeCell ref="A11:B11"/>
     <mergeCell ref="A3:D3"/>
@@ -3831,12 +3843,6 @@
     <mergeCell ref="A14:D14"/>
     <mergeCell ref="A12:B12"/>
     <mergeCell ref="A4:B4"/>
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A9:D9"/>
-    <mergeCell ref="A16:B16"/>
-    <mergeCell ref="A18:D18"/>
-    <mergeCell ref="A15:B15"/>
-    <mergeCell ref="A7:B7"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -3897,7 +3903,7 @@
       <c r="D3" s="57"/>
     </row>
     <row r="4" spans="1:4" ht="22.35" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="66" t="s">
+      <c r="A4" s="63" t="s">
         <v>413</v>
       </c>
       <c r="B4" s="64"/>
@@ -3961,7 +3967,7 @@
       <c r="C11" s="11"/>
     </row>
     <row r="12" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="65" t="s">
+      <c r="A12" s="66" t="s">
         <v>419</v>
       </c>
       <c r="B12" s="64"/>
@@ -4044,7 +4050,7 @@
       <c r="C21" s="11"/>
     </row>
     <row r="22" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="65" t="s">
+      <c r="A22" s="66" t="s">
         <v>426</v>
       </c>
       <c r="B22" s="64"/>
@@ -4233,7 +4239,7 @@
       </c>
     </row>
     <row r="11" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="65" t="s">
+      <c r="A11" s="66" t="s">
         <v>441</v>
       </c>
       <c r="B11" s="64"/>
@@ -4241,7 +4247,7 @@
       <c r="D11" s="64"/>
     </row>
     <row r="12" spans="1:4" ht="22.35" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="66" t="s">
+      <c r="A12" s="63" t="s">
         <v>442</v>
       </c>
       <c r="B12" s="64"/>
@@ -4267,12 +4273,17 @@
       </c>
     </row>
     <row r="15" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="11"/>
-      <c r="B15" s="11"/>
-      <c r="C15" s="11"/>
+      <c r="A15" s="70" t="s">
+        <v>538</v>
+      </c>
+      <c r="B15" s="69"/>
+      <c r="C15" s="34"/>
+      <c r="D15" t="s">
+        <v>539</v>
+      </c>
     </row>
     <row r="16" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="65" t="s">
+      <c r="A16" s="66" t="s">
         <v>446</v>
       </c>
       <c r="B16" s="64"/>
@@ -4317,18 +4328,19 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="11">
-    <mergeCell ref="A13:B13"/>
-    <mergeCell ref="A14:B14"/>
-    <mergeCell ref="A16:D16"/>
-    <mergeCell ref="A11:D11"/>
-    <mergeCell ref="A8:B8"/>
+  <mergeCells count="12">
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A7:B7"/>
     <mergeCell ref="A12:D12"/>
     <mergeCell ref="A3:D3"/>
     <mergeCell ref="A5:B5"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="A16:D16"/>
+    <mergeCell ref="A11:D11"/>
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="A15:B15"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -5272,7 +5284,7 @@
       <c r="D2" s="57"/>
     </row>
     <row r="4" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="65" t="s">
+      <c r="A4" s="66" t="s">
         <v>46</v>
       </c>
       <c r="B4" s="64"/>
@@ -5320,7 +5332,7 @@
       <c r="B9" s="11"/>
     </row>
     <row r="10" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="65" t="s">
+      <c r="A10" s="66" t="s">
         <v>51</v>
       </c>
       <c r="B10" s="64"/>
@@ -5362,7 +5374,7 @@
       <c r="B14" s="11"/>
     </row>
     <row r="15" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="65" t="s">
+      <c r="A15" s="66" t="s">
         <v>56</v>
       </c>
       <c r="B15" s="64"/>
@@ -5467,7 +5479,7 @@
       <c r="B26" s="11"/>
     </row>
     <row r="27" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="65" t="s">
+      <c r="A27" s="66" t="s">
         <v>68</v>
       </c>
       <c r="B27" s="64"/>
@@ -5544,7 +5556,7 @@
       <c r="B35" s="11"/>
     </row>
     <row r="36" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="65" t="s">
+      <c r="A36" s="66" t="s">
         <v>76</v>
       </c>
       <c r="B36" s="64"/>
@@ -5637,7 +5649,7 @@
       <c r="B46" s="11"/>
     </row>
     <row r="47" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="65" t="s">
+      <c r="A47" s="66" t="s">
         <v>86</v>
       </c>
       <c r="B47" s="64"/>
@@ -5703,7 +5715,7 @@
       <c r="B54" s="11"/>
     </row>
     <row r="55" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A55" s="65" t="s">
+      <c r="A55" s="66" t="s">
         <v>93</v>
       </c>
       <c r="B55" s="64"/>
@@ -5711,7 +5723,7 @@
       <c r="D55" s="64"/>
     </row>
     <row r="56" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A56" s="63" t="str">
+      <c r="A56" s="65" t="str">
         <f>IF(B18&gt;0,"• Passive income is grinding the SBD limit — consider moving investments to a holding company or reducing corporate investment income.","")</f>
         <v>• Passive income is grinding the SBD limit — consider moving investments to a holding company or reducing corporate investment income.</v>
       </c>
@@ -5720,7 +5732,7 @@
       <c r="D56" s="64"/>
     </row>
     <row r="57" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A57" s="63" t="str">
+      <c r="A57" s="65" t="str">
         <f>IF(COUNTIF('8. Shareholders &amp; TOSI'!I5:I20,"Not Excluded - TOSI Risk")&gt;0,"• One or more shareholders flagged for TOSI risk — dividends to them may be taxed at top marginal rate.","")</f>
         <v>• One or more shareholders flagged for TOSI risk — dividends to them may be taxed at top marginal rate.</v>
       </c>
@@ -5729,7 +5741,7 @@
       <c r="D57" s="64"/>
     </row>
     <row r="58" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A58" s="63" t="str">
+      <c r="A58" s="65" t="str">
         <f>IF(B44&gt;0,"• Unused Capital Dividend Account balance — a tax-free capital dividend may be available.","")</f>
         <v>• Unused Capital Dividend Account balance — a tax-free capital dividend may be available.</v>
       </c>
@@ -5738,7 +5750,7 @@
       <c r="D58" s="64"/>
     </row>
     <row r="59" spans="1:4" ht="22.35" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A59" s="66" t="s">
+      <c r="A59" s="63" t="s">
         <v>94</v>
       </c>
       <c r="B59" s="64"/>
@@ -5747,12 +5759,6 @@
     </row>
   </sheetData>
   <mergeCells count="13">
-    <mergeCell ref="A59:D59"/>
-    <mergeCell ref="A57:D57"/>
-    <mergeCell ref="A2:D2"/>
-    <mergeCell ref="A10:D10"/>
-    <mergeCell ref="A36:D36"/>
-    <mergeCell ref="A47:D47"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A56:D56"/>
     <mergeCell ref="A27:D27"/>
@@ -5760,6 +5766,12 @@
     <mergeCell ref="A4:D4"/>
     <mergeCell ref="A55:D55"/>
     <mergeCell ref="A15:D15"/>
+    <mergeCell ref="A59:D59"/>
+    <mergeCell ref="A57:D57"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A10:D10"/>
+    <mergeCell ref="A36:D36"/>
+    <mergeCell ref="A47:D47"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -6007,6 +6019,18 @@
     </row>
   </sheetData>
   <mergeCells count="24">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A21:B21"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="A20:B20"/>
+    <mergeCell ref="A11:B11"/>
+    <mergeCell ref="A10:D10"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="A7:B7"/>
     <mergeCell ref="A27:D27"/>
     <mergeCell ref="A29:B29"/>
     <mergeCell ref="A19:B19"/>
@@ -6019,18 +6043,6 @@
     <mergeCell ref="A12:B12"/>
     <mergeCell ref="A23:D23"/>
     <mergeCell ref="A24:B24"/>
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A21:B21"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="A17:B17"/>
-    <mergeCell ref="A8:B8"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="A20:B20"/>
-    <mergeCell ref="A11:B11"/>
-    <mergeCell ref="A10:D10"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="A16:B16"/>
-    <mergeCell ref="A7:B7"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -6404,7 +6416,7 @@
       </c>
     </row>
     <row r="4" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="65" t="s">
+      <c r="A4" s="66" t="s">
         <v>154</v>
       </c>
       <c r="B4" s="64"/>
@@ -6449,7 +6461,7 @@
       <c r="B10" s="11"/>
     </row>
     <row r="11" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="65" t="s">
+      <c r="A11" s="66" t="s">
         <v>158</v>
       </c>
       <c r="B11" s="64"/>
@@ -6491,7 +6503,7 @@
       <c r="B16" s="11"/>
     </row>
     <row r="17" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="65" t="s">
+      <c r="A17" s="66" t="s">
         <v>162</v>
       </c>
       <c r="B17" s="64"/>
@@ -6623,7 +6635,7 @@
       <c r="B33" s="11"/>
     </row>
     <row r="34" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="65" t="s">
+      <c r="A34" s="66" t="s">
         <v>178</v>
       </c>
       <c r="B34" s="64"/>
@@ -6743,7 +6755,7 @@
       <c r="B45" s="11"/>
     </row>
     <row r="46" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="65" t="s">
+      <c r="A46" s="66" t="s">
         <v>193</v>
       </c>
       <c r="B46" s="64"/>
@@ -6967,7 +6979,7 @@
       </c>
     </row>
     <row r="4" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="65" t="s">
+      <c r="A4" s="66" t="s">
         <v>224</v>
       </c>
       <c r="B4" s="64"/>
@@ -7072,7 +7084,7 @@
       <c r="B16" s="33"/>
     </row>
     <row r="17" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="65" t="s">
+      <c r="A17" s="66" t="s">
         <v>238</v>
       </c>
       <c r="B17" s="64"/>
@@ -7163,7 +7175,7 @@
       <c r="B28" s="33"/>
     </row>
     <row r="29" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="65" t="s">
+      <c r="A29" s="66" t="s">
         <v>249</v>
       </c>
       <c r="B29" s="64"/>
@@ -7239,7 +7251,7 @@
       <c r="B38" s="33"/>
     </row>
     <row r="39" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="65" t="s">
+      <c r="A39" s="66" t="s">
         <v>257</v>
       </c>
       <c r="B39" s="64"/>
@@ -7311,7 +7323,7 @@
       <c r="D2" s="57"/>
     </row>
     <row r="4" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="65" t="s">
+      <c r="A4" s="66" t="s">
         <v>264</v>
       </c>
       <c r="B4" s="64"/>
@@ -7348,7 +7360,7 @@
       <c r="C7" s="11"/>
     </row>
     <row r="8" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="65" t="s">
+      <c r="A8" s="66" t="s">
         <v>268</v>
       </c>
       <c r="B8" s="64"/>
@@ -7373,7 +7385,7 @@
       <c r="C10" s="11"/>
     </row>
     <row r="11" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="65" t="s">
+      <c r="A11" s="66" t="s">
         <v>271</v>
       </c>
       <c r="B11" s="64"/>
@@ -7398,7 +7410,7 @@
       <c r="C13" s="11"/>
     </row>
     <row r="14" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="65" t="s">
+      <c r="A14" s="66" t="s">
         <v>274</v>
       </c>
       <c r="B14" s="64"/>
@@ -7461,7 +7473,7 @@
       <c r="C20" s="11"/>
     </row>
     <row r="21" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="65" t="s">
+      <c r="A21" s="66" t="s">
         <v>277</v>
       </c>
       <c r="B21" s="64"/>
@@ -7496,7 +7508,7 @@
       <c r="C25" s="11"/>
     </row>
     <row r="26" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="65" t="s">
+      <c r="A26" s="66" t="s">
         <v>278</v>
       </c>
       <c r="B26" s="64"/>
@@ -7535,6 +7547,12 @@
     </row>
   </sheetData>
   <mergeCells count="14">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A8:D8"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="A26:D26"/>
+    <mergeCell ref="A21:D21"/>
+    <mergeCell ref="A5:B5"/>
     <mergeCell ref="A28:B28"/>
     <mergeCell ref="A2:D2"/>
     <mergeCell ref="A11:D11"/>
@@ -7543,12 +7561,6 @@
     <mergeCell ref="A6:B6"/>
     <mergeCell ref="A14:D14"/>
     <mergeCell ref="A12:B12"/>
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A8:D8"/>
-    <mergeCell ref="A4:D4"/>
-    <mergeCell ref="A26:D26"/>
-    <mergeCell ref="A21:D21"/>
-    <mergeCell ref="A5:B5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>